<commit_message>
feat: expand LO3 RISE prompt engineering
</commit_message>
<xml_diff>
--- a/courseware/Labs/Lab-01-SPC/Worked-Reference.xlsx
+++ b/courseware/Labs/Lab-01-SPC/Worked-Reference.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="65" uniqueCount="49">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="59">
   <si>
     <t xml:space="preserve">Lab 1 - Use Copilot in Excel to create an SPC review</t>
   </si>
@@ -146,6 +146,36 @@
   </si>
   <si>
     <t xml:space="preserve">A baseline mean near 62.0 L/h, calculated limits, three low monitoring signals (T09, T10 and T12), and a short cautious interpretation.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RISE prompt builder</t>
+  </si>
+  <si>
+    <t xml:space="preserve">What this part does</t>
+  </si>
+  <si>
+    <t xml:space="preserve">R - Role</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Engineering data assistant</t>
+  </si>
+  <si>
+    <t xml:space="preserve">I - Input</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Only PumpReadings; eight Baseline and four Monitoring rows</t>
+  </si>
+  <si>
+    <t xml:space="preserve">S - Steps</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Calculate mean, standard deviation and limits; flag rows; create chart</t>
+  </si>
+  <si>
+    <t xml:space="preserve">E - Expectations</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Show formulas; three sentences; no root-cause or safety claim</t>
   </si>
   <si>
     <t xml:space="preserve">Metric</t>
@@ -180,7 +210,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.00"/>
   </numFmts>
-  <fonts count="13">
+  <fonts count="15">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -244,6 +274,21 @@
       <b val="true"/>
       <sz val="14"/>
       <color rgb="FFFFFFFF"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <color rgb="FF087F8C"/>
+      <name val="Arial"/>
+      <family val="0"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF142C3E"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -323,12 +368,16 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="13">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -348,8 +397,20 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
@@ -530,23 +591,27 @@
           </c:marker>
           <c:dLbls>
             <c:txPr>
-              <a:bodyPr wrap="none"/>
+              <a:bodyPr wrap="square"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="r"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
             <c:showSerName val="0"/>
             <c:showPercent val="0"/>
-            <c:separator> </c:separator>
+            <c:separator>; </c:separator>
             <c:showLeaderLines val="1"/>
             <c:leaderLines>
               <c:spPr>
@@ -684,23 +749,27 @@
           </c:marker>
           <c:dLbls>
             <c:txPr>
-              <a:bodyPr wrap="none"/>
+              <a:bodyPr wrap="square"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="r"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
             <c:showSerName val="0"/>
             <c:showPercent val="0"/>
-            <c:separator> </c:separator>
+            <c:separator>; </c:separator>
             <c:showLeaderLines val="1"/>
             <c:leaderLines>
               <c:spPr>
@@ -838,23 +907,27 @@
           </c:marker>
           <c:dLbls>
             <c:txPr>
-              <a:bodyPr wrap="none"/>
+              <a:bodyPr wrap="square"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="r"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
             <c:showSerName val="0"/>
             <c:showPercent val="0"/>
-            <c:separator> </c:separator>
+            <c:separator>; </c:separator>
             <c:showLeaderLines val="1"/>
             <c:leaderLines>
               <c:spPr>
@@ -992,23 +1065,27 @@
           </c:marker>
           <c:dLbls>
             <c:txPr>
-              <a:bodyPr wrap="none"/>
+              <a:bodyPr wrap="square"/>
               <a:lstStyle/>
               <a:p>
                 <a:pPr>
                   <a:defRPr sz="1000" b="0" u="none" strike="noStrike">
+                    <a:solidFill>
+                      <a:srgbClr val="000000"/>
+                    </a:solidFill>
                     <a:uFillTx/>
                     <a:latin typeface="Arial"/>
                   </a:defRPr>
                 </a:pPr>
               </a:p>
             </c:txPr>
+            <c:dLblPos val="r"/>
             <c:showLegendKey val="0"/>
             <c:showVal val="0"/>
             <c:showCatName val="0"/>
             <c:showSerName val="0"/>
             <c:showPercent val="0"/>
-            <c:separator> </c:separator>
+            <c:separator>; </c:separator>
             <c:showLeaderLines val="1"/>
             <c:leaderLines>
               <c:spPr>
@@ -1124,11 +1201,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="2806279"/>
-        <c:axId val="3799632"/>
+        <c:axId val="45376181"/>
+        <c:axId val="59829899"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="2806279"/>
+        <c:axId val="45376181"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1167,7 +1244,7 @@
             </a:ln>
           </c:spPr>
         </c:title>
-        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:numFmt formatCode="General" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1194,7 +1271,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="3799632"/>
+        <c:crossAx val="59829899"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1202,7 +1279,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="3799632"/>
+        <c:axId val="59829899"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1251,7 +1328,7 @@
             </a:ln>
           </c:spPr>
         </c:title>
-        <c:numFmt formatCode="0.00" sourceLinked="1"/>
+        <c:numFmt formatCode="0.00" sourceLinked="0"/>
         <c:majorTickMark val="none"/>
         <c:minorTickMark val="none"/>
         <c:tickLblPos val="nextTo"/>
@@ -1278,7 +1355,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2806279"/>
+        <c:crossAx val="45376181"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -1560,9 +1637,9 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>17</xdr:col>
-      <xdr:colOff>256320</xdr:colOff>
+      <xdr:colOff>255960</xdr:colOff>
       <xdr:row>14</xdr:row>
-      <xdr:rowOff>6120</xdr:rowOff>
+      <xdr:rowOff>5760</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame>
       <xdr:nvGraphicFramePr>
@@ -1571,7 +1648,7 @@
       </xdr:nvGraphicFramePr>
       <xdr:xfrm>
         <a:off x="7660080" y="190440"/>
-        <a:ext cx="5759640" cy="2879640"/>
+        <a:ext cx="5759280" cy="2872800"/>
       </xdr:xfrm>
       <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
@@ -1778,85 +1855,85 @@
   <dimension ref="A1:B10"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="105"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="105"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="22.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="1" t="s">
+    <row r="1" customFormat="false" ht="21.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1"/>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
+      <c r="B1" s="2"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="4" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="B3" s="3" t="s">
+      <c r="B3" s="4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B4" s="3" t="s">
+      <c r="B4" s="4" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="2" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="3" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="B5" s="4" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="2" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="4" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="2" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="4" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="2" t="s">
+    <row r="8" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="B9" s="3" t="s">
+      <c r="B9" s="4" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="2" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="B10" s="4" t="s">
         <v>18</v>
       </c>
     </row>
@@ -1882,151 +1959,151 @@
   <dimension ref="A1:C13"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="18"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="4" t="s">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="B1" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="C1" s="4" t="s">
+      <c r="C1" s="5" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="5" t="s">
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B2" s="5" t="s">
+      <c r="B2" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="C2" s="5" t="n">
+      <c r="C2" s="6" t="n">
         <v>61.8</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="5" t="s">
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="6" t="s">
         <v>24</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="C3" s="5" t="n">
+      <c r="C3" s="6" t="n">
         <v>62.1</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B4" s="5" t="s">
+      <c r="B4" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="C4" s="5" t="n">
+      <c r="C4" s="6" t="n">
         <v>61.9</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="C5" s="5" t="n">
+      <c r="C5" s="6" t="n">
         <v>62.2</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="B6" s="5" t="s">
+      <c r="B6" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="C6" s="5" t="n">
+      <c r="C6" s="6" t="n">
         <v>62</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="5" t="s">
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="6" t="s">
         <v>28</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="C7" s="5" t="n">
+      <c r="C7" s="6" t="n">
         <v>61.7</v>
       </c>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="B8" s="5" t="s">
+      <c r="B8" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="C8" s="5" t="n">
+      <c r="C8" s="6" t="n">
         <v>62.3</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="s">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6" t="s">
         <v>30</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="6" t="s">
         <v>23</v>
       </c>
-      <c r="C9" s="5" t="n">
+      <c r="C9" s="6" t="n">
         <v>62</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5" t="s">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B10" s="5" t="s">
+      <c r="B10" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="C10" s="5" t="n">
+      <c r="C10" s="6" t="n">
         <v>59.6</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5" t="s">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="C11" s="5" t="n">
+      <c r="C11" s="6" t="n">
         <v>59.4</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="5" t="s">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="B12" s="5" t="s">
+      <c r="B12" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="C12" s="5" t="n">
+      <c r="C12" s="6" t="n">
         <v>62.1</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5" t="s">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="B13" s="5" t="s">
+      <c r="B13" s="6" t="s">
         <v>32</v>
       </c>
-      <c r="C13" s="5" t="n">
+      <c r="C13" s="6" t="n">
         <v>59.5</v>
       </c>
     </row>
@@ -2049,40 +2126,81 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="true"/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="120"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="90"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="6" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="7" t="s">
         <v>36</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="81.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+      <c r="A2" s="4" t="s">
         <v>37</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="6" t="s">
+    <row r="3" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="7" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="3" t="s">
+      <c r="A4" s="4" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="6" t="s">
+    <row r="5" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="7" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="4" t="s">
         <v>40</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="8" t="s">
+        <v>41</v>
+      </c>
+      <c r="B8" s="8" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="B9" s="10" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="9" t="s">
+        <v>45</v>
+      </c>
+      <c r="B10" s="10" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="9" t="s">
+        <v>47</v>
+      </c>
+      <c r="B11" s="10" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="B12" s="10" t="s">
+        <v>50</v>
       </c>
     </row>
   </sheetData>
@@ -2104,471 +2222,471 @@
   <dimension ref="A1:G19"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="13"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="15"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="13"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="15"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="5" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="18"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="B1" s="4" t="s">
-        <v>42</v>
-      </c>
-      <c r="C1" s="4"/>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
-      <c r="F1" s="4"/>
-      <c r="G1" s="4"/>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="B2" s="7" t="n">
+    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="B1" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="B2" s="11" t="n">
         <f aca="false">AVERAGE(Pump_Readings!C2:C9)</f>
         <v>62</v>
       </c>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-    </row>
-    <row r="3" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="5" t="s">
-        <v>44</v>
-      </c>
-      <c r="B3" s="7" t="n">
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="6"/>
+      <c r="G2" s="6"/>
+    </row>
+    <row r="3" customFormat="false" ht="45.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A3" s="6" t="s">
+        <v>54</v>
+      </c>
+      <c r="B3" s="11" t="n">
         <f aca="false">STDEV(Pump_Readings!C2:C9)</f>
         <v>0.2</v>
       </c>
-      <c r="C3" s="5"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5"/>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="B4" s="7" t="n">
+      <c r="C3" s="6"/>
+      <c r="D3" s="6"/>
+      <c r="E3" s="6"/>
+      <c r="F3" s="6"/>
+      <c r="G3" s="6"/>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="6" t="s">
+        <v>55</v>
+      </c>
+      <c r="B4" s="11" t="n">
         <f aca="false">B2+3*B3</f>
         <v>62.6</v>
       </c>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5"/>
-      <c r="G4" s="5"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="B5" s="7" t="n">
+      <c r="C4" s="6"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
+      <c r="F4" s="6"/>
+      <c r="G4" s="6"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="6" t="s">
+        <v>56</v>
+      </c>
+      <c r="B5" s="11" t="n">
         <f aca="false">B2-3*B3</f>
         <v>61.4</v>
       </c>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5"/>
-      <c r="B6" s="5"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
-      <c r="F6" s="5"/>
-      <c r="G6" s="5"/>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="8" t="s">
+      <c r="C5" s="6"/>
+      <c r="D5" s="6"/>
+      <c r="E5" s="6"/>
+      <c r="F5" s="6"/>
+      <c r="G5" s="6"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="6"/>
+      <c r="B6" s="6"/>
+      <c r="C6" s="6"/>
+      <c r="D6" s="6"/>
+      <c r="E6" s="6"/>
+      <c r="F6" s="6"/>
+      <c r="G6" s="6"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="8" t="s">
+      <c r="B7" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="C7" s="8" t="s">
+      <c r="C7" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="D7" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="E7" s="8" t="s">
-        <v>45</v>
-      </c>
-      <c r="F7" s="8" t="s">
-        <v>46</v>
-      </c>
-      <c r="G7" s="8" t="s">
-        <v>48</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="str">
+      <c r="D7" s="12" t="s">
+        <v>57</v>
+      </c>
+      <c r="E7" s="12" t="s">
+        <v>55</v>
+      </c>
+      <c r="F7" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="G7" s="12" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="6" t="str">
         <f aca="false">Pump_Readings!A2</f>
         <v>T01</v>
       </c>
-      <c r="B8" s="5" t="str">
+      <c r="B8" s="6" t="str">
         <f aca="false">Pump_Readings!B2</f>
         <v>Baseline</v>
       </c>
-      <c r="C8" s="5" t="n">
+      <c r="C8" s="6" t="n">
         <f aca="false">Pump_Readings!C2</f>
         <v>61.8</v>
       </c>
-      <c r="D8" s="7" t="n">
+      <c r="D8" s="11" t="n">
         <f aca="false">$B$2</f>
         <v>62</v>
       </c>
-      <c r="E8" s="7" t="n">
+      <c r="E8" s="11" t="n">
         <f aca="false">$B$4</f>
         <v>62.6</v>
       </c>
-      <c r="F8" s="7" t="n">
+      <c r="F8" s="11" t="n">
         <f aca="false">$B$5</f>
         <v>61.4</v>
       </c>
-      <c r="G8" s="5" t="str">
+      <c r="G8" s="6" t="str">
         <f aca="false">IF(B8="Baseline","Reference",IF(C8&lt;F8,"Below LCL",IF(C8&gt;E8,"Above UCL","Within limits")))</f>
         <v>Reference</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="5" t="str">
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="6" t="str">
         <f aca="false">Pump_Readings!A3</f>
         <v>T02</v>
       </c>
-      <c r="B9" s="5" t="str">
+      <c r="B9" s="6" t="str">
         <f aca="false">Pump_Readings!B3</f>
         <v>Baseline</v>
       </c>
-      <c r="C9" s="5" t="n">
+      <c r="C9" s="6" t="n">
         <f aca="false">Pump_Readings!C3</f>
         <v>62.1</v>
       </c>
-      <c r="D9" s="7" t="n">
+      <c r="D9" s="11" t="n">
         <f aca="false">$B$2</f>
         <v>62</v>
       </c>
-      <c r="E9" s="7" t="n">
+      <c r="E9" s="11" t="n">
         <f aca="false">$B$4</f>
         <v>62.6</v>
       </c>
-      <c r="F9" s="7" t="n">
+      <c r="F9" s="11" t="n">
         <f aca="false">$B$5</f>
         <v>61.4</v>
       </c>
-      <c r="G9" s="5" t="str">
+      <c r="G9" s="6" t="str">
         <f aca="false">IF(B9="Baseline","Reference",IF(C9&lt;F9,"Below LCL",IF(C9&gt;E9,"Above UCL","Within limits")))</f>
         <v>Reference</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="5" t="str">
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A10" s="6" t="str">
         <f aca="false">Pump_Readings!A4</f>
         <v>T03</v>
       </c>
-      <c r="B10" s="5" t="str">
+      <c r="B10" s="6" t="str">
         <f aca="false">Pump_Readings!B4</f>
         <v>Baseline</v>
       </c>
-      <c r="C10" s="5" t="n">
+      <c r="C10" s="6" t="n">
         <f aca="false">Pump_Readings!C4</f>
         <v>61.9</v>
       </c>
-      <c r="D10" s="7" t="n">
+      <c r="D10" s="11" t="n">
         <f aca="false">$B$2</f>
         <v>62</v>
       </c>
-      <c r="E10" s="7" t="n">
+      <c r="E10" s="11" t="n">
         <f aca="false">$B$4</f>
         <v>62.6</v>
       </c>
-      <c r="F10" s="7" t="n">
+      <c r="F10" s="11" t="n">
         <f aca="false">$B$5</f>
         <v>61.4</v>
       </c>
-      <c r="G10" s="5" t="str">
+      <c r="G10" s="6" t="str">
         <f aca="false">IF(B10="Baseline","Reference",IF(C10&lt;F10,"Below LCL",IF(C10&gt;E10,"Above UCL","Within limits")))</f>
         <v>Reference</v>
       </c>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="5" t="str">
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="6" t="str">
         <f aca="false">Pump_Readings!A5</f>
         <v>T04</v>
       </c>
-      <c r="B11" s="5" t="str">
+      <c r="B11" s="6" t="str">
         <f aca="false">Pump_Readings!B5</f>
         <v>Baseline</v>
       </c>
-      <c r="C11" s="5" t="n">
+      <c r="C11" s="6" t="n">
         <f aca="false">Pump_Readings!C5</f>
         <v>62.2</v>
       </c>
-      <c r="D11" s="7" t="n">
+      <c r="D11" s="11" t="n">
         <f aca="false">$B$2</f>
         <v>62</v>
       </c>
-      <c r="E11" s="7" t="n">
+      <c r="E11" s="11" t="n">
         <f aca="false">$B$4</f>
         <v>62.6</v>
       </c>
-      <c r="F11" s="7" t="n">
+      <c r="F11" s="11" t="n">
         <f aca="false">$B$5</f>
         <v>61.4</v>
       </c>
-      <c r="G11" s="5" t="str">
+      <c r="G11" s="6" t="str">
         <f aca="false">IF(B11="Baseline","Reference",IF(C11&lt;F11,"Below LCL",IF(C11&gt;E11,"Above UCL","Within limits")))</f>
         <v>Reference</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="5" t="str">
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="6" t="str">
         <f aca="false">Pump_Readings!A6</f>
         <v>T05</v>
       </c>
-      <c r="B12" s="5" t="str">
+      <c r="B12" s="6" t="str">
         <f aca="false">Pump_Readings!B6</f>
         <v>Baseline</v>
       </c>
-      <c r="C12" s="5" t="n">
+      <c r="C12" s="6" t="n">
         <f aca="false">Pump_Readings!C6</f>
         <v>62</v>
       </c>
-      <c r="D12" s="7" t="n">
+      <c r="D12" s="11" t="n">
         <f aca="false">$B$2</f>
         <v>62</v>
       </c>
-      <c r="E12" s="7" t="n">
+      <c r="E12" s="11" t="n">
         <f aca="false">$B$4</f>
         <v>62.6</v>
       </c>
-      <c r="F12" s="7" t="n">
+      <c r="F12" s="11" t="n">
         <f aca="false">$B$5</f>
         <v>61.4</v>
       </c>
-      <c r="G12" s="5" t="str">
+      <c r="G12" s="6" t="str">
         <f aca="false">IF(B12="Baseline","Reference",IF(C12&lt;F12,"Below LCL",IF(C12&gt;E12,"Above UCL","Within limits")))</f>
         <v>Reference</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5" t="str">
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="6" t="str">
         <f aca="false">Pump_Readings!A7</f>
         <v>T06</v>
       </c>
-      <c r="B13" s="5" t="str">
+      <c r="B13" s="6" t="str">
         <f aca="false">Pump_Readings!B7</f>
         <v>Baseline</v>
       </c>
-      <c r="C13" s="5" t="n">
+      <c r="C13" s="6" t="n">
         <f aca="false">Pump_Readings!C7</f>
         <v>61.7</v>
       </c>
-      <c r="D13" s="7" t="n">
+      <c r="D13" s="11" t="n">
         <f aca="false">$B$2</f>
         <v>62</v>
       </c>
-      <c r="E13" s="7" t="n">
+      <c r="E13" s="11" t="n">
         <f aca="false">$B$4</f>
         <v>62.6</v>
       </c>
-      <c r="F13" s="7" t="n">
+      <c r="F13" s="11" t="n">
         <f aca="false">$B$5</f>
         <v>61.4</v>
       </c>
-      <c r="G13" s="5" t="str">
+      <c r="G13" s="6" t="str">
         <f aca="false">IF(B13="Baseline","Reference",IF(C13&lt;F13,"Below LCL",IF(C13&gt;E13,"Above UCL","Within limits")))</f>
         <v>Reference</v>
       </c>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5" t="str">
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="6" t="str">
         <f aca="false">Pump_Readings!A8</f>
         <v>T07</v>
       </c>
-      <c r="B14" s="5" t="str">
+      <c r="B14" s="6" t="str">
         <f aca="false">Pump_Readings!B8</f>
         <v>Baseline</v>
       </c>
-      <c r="C14" s="5" t="n">
+      <c r="C14" s="6" t="n">
         <f aca="false">Pump_Readings!C8</f>
         <v>62.3</v>
       </c>
-      <c r="D14" s="7" t="n">
+      <c r="D14" s="11" t="n">
         <f aca="false">$B$2</f>
         <v>62</v>
       </c>
-      <c r="E14" s="7" t="n">
+      <c r="E14" s="11" t="n">
         <f aca="false">$B$4</f>
         <v>62.6</v>
       </c>
-      <c r="F14" s="7" t="n">
+      <c r="F14" s="11" t="n">
         <f aca="false">$B$5</f>
         <v>61.4</v>
       </c>
-      <c r="G14" s="5" t="str">
+      <c r="G14" s="6" t="str">
         <f aca="false">IF(B14="Baseline","Reference",IF(C14&lt;F14,"Below LCL",IF(C14&gt;E14,"Above UCL","Within limits")))</f>
         <v>Reference</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="5" t="str">
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="6" t="str">
         <f aca="false">Pump_Readings!A9</f>
         <v>T08</v>
       </c>
-      <c r="B15" s="5" t="str">
+      <c r="B15" s="6" t="str">
         <f aca="false">Pump_Readings!B9</f>
         <v>Baseline</v>
       </c>
-      <c r="C15" s="5" t="n">
+      <c r="C15" s="6" t="n">
         <f aca="false">Pump_Readings!C9</f>
         <v>62</v>
       </c>
-      <c r="D15" s="7" t="n">
+      <c r="D15" s="11" t="n">
         <f aca="false">$B$2</f>
         <v>62</v>
       </c>
-      <c r="E15" s="7" t="n">
+      <c r="E15" s="11" t="n">
         <f aca="false">$B$4</f>
         <v>62.6</v>
       </c>
-      <c r="F15" s="7" t="n">
+      <c r="F15" s="11" t="n">
         <f aca="false">$B$5</f>
         <v>61.4</v>
       </c>
-      <c r="G15" s="5" t="str">
+      <c r="G15" s="6" t="str">
         <f aca="false">IF(B15="Baseline","Reference",IF(C15&lt;F15,"Below LCL",IF(C15&gt;E15,"Above UCL","Within limits")))</f>
         <v>Reference</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="5" t="str">
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A16" s="6" t="str">
         <f aca="false">Pump_Readings!A10</f>
         <v>T09</v>
       </c>
-      <c r="B16" s="5" t="str">
+      <c r="B16" s="6" t="str">
         <f aca="false">Pump_Readings!B10</f>
         <v>Monitoring</v>
       </c>
-      <c r="C16" s="5" t="n">
+      <c r="C16" s="6" t="n">
         <f aca="false">Pump_Readings!C10</f>
         <v>59.6</v>
       </c>
-      <c r="D16" s="7" t="n">
+      <c r="D16" s="11" t="n">
         <f aca="false">$B$2</f>
         <v>62</v>
       </c>
-      <c r="E16" s="7" t="n">
+      <c r="E16" s="11" t="n">
         <f aca="false">$B$4</f>
         <v>62.6</v>
       </c>
-      <c r="F16" s="7" t="n">
+      <c r="F16" s="11" t="n">
         <f aca="false">$B$5</f>
         <v>61.4</v>
       </c>
-      <c r="G16" s="5" t="str">
+      <c r="G16" s="6" t="str">
         <f aca="false">IF(B16="Baseline","Reference",IF(C16&lt;F16,"Below LCL",IF(C16&gt;E16,"Above UCL","Within limits")))</f>
         <v>Below LCL</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="5" t="str">
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A17" s="6" t="str">
         <f aca="false">Pump_Readings!A11</f>
         <v>T10</v>
       </c>
-      <c r="B17" s="5" t="str">
+      <c r="B17" s="6" t="str">
         <f aca="false">Pump_Readings!B11</f>
         <v>Monitoring</v>
       </c>
-      <c r="C17" s="5" t="n">
+      <c r="C17" s="6" t="n">
         <f aca="false">Pump_Readings!C11</f>
         <v>59.4</v>
       </c>
-      <c r="D17" s="7" t="n">
+      <c r="D17" s="11" t="n">
         <f aca="false">$B$2</f>
         <v>62</v>
       </c>
-      <c r="E17" s="7" t="n">
+      <c r="E17" s="11" t="n">
         <f aca="false">$B$4</f>
         <v>62.6</v>
       </c>
-      <c r="F17" s="7" t="n">
+      <c r="F17" s="11" t="n">
         <f aca="false">$B$5</f>
         <v>61.4</v>
       </c>
-      <c r="G17" s="5" t="str">
+      <c r="G17" s="6" t="str">
         <f aca="false">IF(B17="Baseline","Reference",IF(C17&lt;F17,"Below LCL",IF(C17&gt;E17,"Above UCL","Within limits")))</f>
         <v>Below LCL</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="5" t="str">
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A18" s="6" t="str">
         <f aca="false">Pump_Readings!A12</f>
         <v>T11</v>
       </c>
-      <c r="B18" s="5" t="str">
+      <c r="B18" s="6" t="str">
         <f aca="false">Pump_Readings!B12</f>
         <v>Monitoring</v>
       </c>
-      <c r="C18" s="5" t="n">
+      <c r="C18" s="6" t="n">
         <f aca="false">Pump_Readings!C12</f>
         <v>62.1</v>
       </c>
-      <c r="D18" s="7" t="n">
+      <c r="D18" s="11" t="n">
         <f aca="false">$B$2</f>
         <v>62</v>
       </c>
-      <c r="E18" s="7" t="n">
+      <c r="E18" s="11" t="n">
         <f aca="false">$B$4</f>
         <v>62.6</v>
       </c>
-      <c r="F18" s="7" t="n">
+      <c r="F18" s="11" t="n">
         <f aca="false">$B$5</f>
         <v>61.4</v>
       </c>
-      <c r="G18" s="5" t="str">
+      <c r="G18" s="6" t="str">
         <f aca="false">IF(B18="Baseline","Reference",IF(C18&lt;F18,"Below LCL",IF(C18&gt;E18,"Above UCL","Within limits")))</f>
         <v>Within limits</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="5" t="str">
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A19" s="6" t="str">
         <f aca="false">Pump_Readings!A13</f>
         <v>T12</v>
       </c>
-      <c r="B19" s="5" t="str">
+      <c r="B19" s="6" t="str">
         <f aca="false">Pump_Readings!B13</f>
         <v>Monitoring</v>
       </c>
-      <c r="C19" s="5" t="n">
+      <c r="C19" s="6" t="n">
         <f aca="false">Pump_Readings!C13</f>
         <v>59.5</v>
       </c>
-      <c r="D19" s="7" t="n">
+      <c r="D19" s="11" t="n">
         <f aca="false">$B$2</f>
         <v>62</v>
       </c>
-      <c r="E19" s="7" t="n">
+      <c r="E19" s="11" t="n">
         <f aca="false">$B$4</f>
         <v>62.6</v>
       </c>
-      <c r="F19" s="7" t="n">
+      <c r="F19" s="11" t="n">
         <f aca="false">$B$5</f>
         <v>61.4</v>
       </c>
-      <c r="G19" s="5" t="str">
+      <c r="G19" s="6" t="str">
         <f aca="false">IF(B19="Baseline","Reference",IF(C19&lt;F19,"Below LCL",IF(C19&gt;E19,"Above UCL","Within limits")))</f>
         <v>Below LCL</v>
       </c>

</xml_diff>